<commit_message>
Update config workbooks for v1.2.0
</commit_message>
<xml_diff>
--- a/config/setup_test_a2700.xlsx
+++ b/config/setup_test_a2700.xlsx
@@ -1,27 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JOYS\Documents\Claude\Projects\vision\VisionOCR\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PNT\61.AI\VisionOCR\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9863AFF-D778-4C7E-B026-97E88E203BC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CDED1AF-9D85-45B3-ACB2-6262435AB975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30552" yWindow="-2832" windowWidth="20196" windowHeight="21456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="-22020" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="setup_cases" sheetId="1" r:id="rId1"/>
     <sheet name="xy" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="202">
   <si>
     <t>name</t>
   </si>
@@ -634,6 +639,66 @@
   </si>
   <si>
     <t>370, 300; 370, 360</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>비밀번호좌표</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rootech0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>150, 370</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>315, 250</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>600, 250</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>370, 250</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>260, 250</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>345, 370</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>425, 310</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>660, 200</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>345, 430</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>엔터</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>340, 400; 295, 455; 320, 300</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>setup; setup; 165, 160; 75, 65</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TRUE; MHN</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1075,27 +1140,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R48"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="3" max="3" width="8.625" customWidth="1"/>
+    <col min="3" max="3" width="8.58203125" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="13.5" customWidth="1"/>
     <col min="6" max="6" width="18.25" customWidth="1"/>
-    <col min="7" max="7" width="14.375" customWidth="1"/>
+    <col min="7" max="7" width="27.25" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.375" customWidth="1"/>
-    <col min="10" max="10" width="13.75" customWidth="1"/>
+    <col min="9" max="9" width="17.33203125" customWidth="1"/>
+    <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="62.125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="26.125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.625" customWidth="1"/>
-    <col min="15" max="15" width="17.125" customWidth="1"/>
+    <col min="12" max="12" width="62.08203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="47.08203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.58203125" customWidth="1"/>
+    <col min="15" max="15" width="17.08203125" customWidth="1"/>
     <col min="16" max="16" width="14.5" customWidth="1"/>
-    <col min="17" max="17" width="16.375" customWidth="1"/>
+    <col min="17" max="17" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1149,7 +1214,7 @@
       </c>
       <c r="R1" s="1"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>17</v>
       </c>
@@ -1203,7 +1268,7 @@
       </c>
       <c r="R2" s="3"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
         <v>34</v>
       </c>
@@ -1221,7 +1286,7 @@
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="8" t="s">
-        <v>38</v>
+        <v>200</v>
       </c>
       <c r="H3" s="9" t="s">
         <v>39</v>
@@ -1229,7 +1294,9 @@
       <c r="I3" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="J3" s="8"/>
+      <c r="J3" s="8" t="s">
+        <v>201</v>
+      </c>
       <c r="K3" s="8" t="s">
         <v>41</v>
       </c>
@@ -1237,7 +1304,7 @@
         <v>42</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>43</v>
+        <v>199</v>
       </c>
       <c r="N3" s="7" t="s">
         <v>44</v>
@@ -1250,7 +1317,7 @@
       </c>
       <c r="Q3" s="8"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
         <v>46</v>
       </c>
@@ -1280,7 +1347,7 @@
         <v>47</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>43</v>
+        <v>199</v>
       </c>
       <c r="N4" s="7" t="s">
         <v>48</v>
@@ -1293,7 +1360,7 @@
       </c>
       <c r="Q4" s="8"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A5" s="8" t="s">
         <v>49</v>
       </c>
@@ -1335,7 +1402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A6" s="8" t="s">
         <v>58</v>
       </c>
@@ -1377,7 +1444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A7" s="8" t="s">
         <v>60</v>
       </c>
@@ -1419,7 +1486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A8" s="8" t="s">
         <v>63</v>
       </c>
@@ -1461,7 +1528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A9" s="8" t="s">
         <v>67</v>
       </c>
@@ -1503,7 +1570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A10" s="8" t="s">
         <v>68</v>
       </c>
@@ -1545,7 +1612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A11" s="8" t="s">
         <v>69</v>
       </c>
@@ -1587,7 +1654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A12" s="8" t="s">
         <v>73</v>
       </c>
@@ -1629,7 +1696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A13" s="8" t="s">
         <v>75</v>
       </c>
@@ -1671,7 +1738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A14" s="8" t="s">
         <v>76</v>
       </c>
@@ -1713,7 +1780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A15" s="8" t="s">
         <v>80</v>
       </c>
@@ -1755,7 +1822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A16" s="8" t="s">
         <v>81</v>
       </c>
@@ -1798,7 +1865,7 @@
       </c>
       <c r="R16" s="10"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A17" s="8" t="s">
         <v>132</v>
       </c>
@@ -1842,7 +1909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A18" s="8" t="s">
         <v>133</v>
       </c>
@@ -1884,7 +1951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A19" s="8" t="s">
         <v>134</v>
       </c>
@@ -1926,7 +1993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A20" s="8" t="s">
         <v>184</v>
       </c>
@@ -1968,7 +2035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A21" s="8" t="s">
         <v>135</v>
       </c>
@@ -2010,7 +2077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A22" s="8" t="s">
         <v>138</v>
       </c>
@@ -2052,7 +2119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A23" s="8" t="s">
         <v>140</v>
       </c>
@@ -2094,7 +2161,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A24" s="8" t="s">
         <v>136</v>
       </c>
@@ -2136,7 +2203,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A25" s="8" t="s">
         <v>142</v>
       </c>
@@ -2178,7 +2245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A26" s="8" t="s">
         <v>143</v>
       </c>
@@ -2220,7 +2287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A27" s="8" t="s">
         <v>146</v>
       </c>
@@ -2262,7 +2329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A28" s="8" t="s">
         <v>147</v>
       </c>
@@ -2304,7 +2371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A29" s="8" t="s">
         <v>137</v>
       </c>
@@ -2346,7 +2413,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A30" s="8" t="s">
         <v>150</v>
       </c>
@@ -2388,7 +2455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A31" s="8" t="s">
         <v>151</v>
       </c>
@@ -2430,7 +2497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A32" s="8" t="s">
         <v>156</v>
       </c>
@@ -2474,7 +2541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A33" s="8" t="s">
         <v>157</v>
       </c>
@@ -2517,7 +2584,7 @@
       </c>
       <c r="R33" s="10"/>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A34" s="8" t="s">
         <v>160</v>
       </c>
@@ -2559,7 +2626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A35" s="8" t="s">
         <v>161</v>
       </c>
@@ -2601,7 +2668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A36" s="8" t="s">
         <v>98</v>
       </c>
@@ -2643,7 +2710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A37" s="8" t="s">
         <v>101</v>
       </c>
@@ -2685,7 +2752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A38" s="8" t="s">
         <v>164</v>
       </c>
@@ -2727,7 +2794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A39" s="8" t="s">
         <v>165</v>
       </c>
@@ -2769,7 +2836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A40" s="8" t="s">
         <v>168</v>
       </c>
@@ -2813,7 +2880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A41" s="8" t="s">
         <v>169</v>
       </c>
@@ -2855,7 +2922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A42" s="8" t="s">
         <v>170</v>
       </c>
@@ -2897,7 +2964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A43" s="8" t="s">
         <v>175</v>
       </c>
@@ -2939,7 +3006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A44" s="8" t="s">
         <v>174</v>
       </c>
@@ -2981,7 +3048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A45" s="8" t="s">
         <v>180</v>
       </c>
@@ -3022,7 +3089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A46" s="8" t="s">
         <v>181</v>
       </c>
@@ -3064,7 +3131,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A47" s="8"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -3082,7 +3149,7 @@
       <c r="O47" s="8"/>
       <c r="P47" s="8"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
       <c r="D48" s="9"/>
@@ -3107,22 +3174,23 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:I15"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:I29"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="14.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9" style="14" customWidth="1"/>
     <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>6</v>
       </c>
@@ -3145,7 +3213,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3174,7 +3242,7 @@
         <v>295455</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2</v>
       </c>
@@ -3197,7 +3265,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3214,7 +3282,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>4</v>
       </c>
@@ -3231,7 +3299,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>5</v>
       </c>
@@ -3245,7 +3313,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="F8" s="14">
         <v>3</v>
       </c>
@@ -3253,7 +3321,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="F9" s="14">
         <v>4</v>
       </c>
@@ -3261,7 +3329,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="F10" s="14">
         <v>5</v>
       </c>
@@ -3269,7 +3337,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="F11" s="14">
         <v>6</v>
       </c>
@@ -3277,7 +3345,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="F12" s="14">
         <v>7</v>
       </c>
@@ -3285,7 +3353,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="F13" s="14">
         <v>8</v>
       </c>
@@ -3293,7 +3361,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="F14" s="14">
         <v>9</v>
       </c>
@@ -3301,17 +3369,83 @@
         <v>185</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="F15" s="14" t="s">
         <v>112</v>
       </c>
       <c r="G15" t="s">
         <v>127</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B18" t="s">
+        <v>187</v>
+      </c>
+      <c r="C18" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C19" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C20" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C21" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C22" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C23" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C24" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C25" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C26" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C27" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="C28" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B29" t="s">
+        <v>198</v>
+      </c>
+      <c r="C29" t="s">
+        <v>197</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>